<commit_message>
- added newly received loss-of-sale source files - prepared data for import into existing sync pipeline - ensured file structure matches current import schema
</commit_message>
<xml_diff>
--- a/data/lossofsale_sg_calicut.xlsx
+++ b/data/lossofsale_sg_calicut.xlsx
@@ -660,20 +660,20 @@
       </c>
       <c t="inlineStr" r="C10">
         <is>
-          <t xml:space="preserve">nihad</t>
+          <t xml:space="preserve">shreyas</t>
         </is>
       </c>
       <c r="D10" s="65">
-        <v>9995874916</v>
+        <v>7994208854</v>
       </c>
       <c t="inlineStr" r="E10">
         <is>
-          <t xml:space="preserve">12-12-2025</t>
+          <t xml:space="preserve">28-12-2025</t>
         </is>
       </c>
       <c t="inlineStr" r="F10">
         <is>
-          <t xml:space="preserve">PUNARTH K</t>
+          <t xml:space="preserve">MUHAMMED ROSHAN C V</t>
         </is>
       </c>
       <c t="inlineStr" r="G10">
@@ -683,12 +683,12 @@
       </c>
       <c t="inlineStr" r="H10">
         <is>
-          <t xml:space="preserve">PRODUCT</t>
+          <t xml:space="preserve">ENQUIRY</t>
         </is>
       </c>
       <c t="inlineStr" r="I10">
         <is>
-          <t xml:space="preserve">REQUIRED MODEL NOT AVAILABLE</t>
+          <t xml:space="preserve">ENQUIRY WITHOUT BRIDE/FAMILY</t>
         </is>
       </c>
       <c t="inlineStr" r="J10">
@@ -698,7 +698,7 @@
       </c>
       <c t="inlineStr" r="K10">
         <is>
-          <t xml:space="preserve">COLLECTION NOT OKAY</t>
+          <t xml:space="preserve">custumer need to visit other store</t>
         </is>
       </c>
     </row>
@@ -708,20 +708,20 @@
       </c>
       <c t="inlineStr" r="B11">
         <is>
-          <t xml:space="preserve">12-12-2025</t>
+          <t xml:space="preserve">13-12-2025</t>
         </is>
       </c>
       <c t="inlineStr" r="C11">
         <is>
-          <t xml:space="preserve">shreyas</t>
+          <t xml:space="preserve">sachin</t>
         </is>
       </c>
       <c r="D11" s="65">
-        <v>7994208854</v>
+        <v>9895964853</v>
       </c>
       <c t="inlineStr" r="E11">
         <is>
-          <t xml:space="preserve">28-12-2025</t>
+          <t xml:space="preserve">30-12-2025</t>
         </is>
       </c>
       <c t="inlineStr" r="F11">
@@ -736,12 +736,12 @@
       </c>
       <c t="inlineStr" r="H11">
         <is>
-          <t xml:space="preserve">ENQUIRY</t>
+          <t xml:space="preserve">PRODUCT</t>
         </is>
       </c>
       <c t="inlineStr" r="I11">
         <is>
-          <t xml:space="preserve">ENQUIRY WITHOUT BRIDE/FAMILY</t>
+          <t xml:space="preserve">PRODUCT NOT AVAILABLE</t>
         </is>
       </c>
       <c t="inlineStr" r="J11">
@@ -751,7 +751,7 @@
       </c>
       <c t="inlineStr" r="K11">
         <is>
-          <t xml:space="preserve">custumer need to visit other store</t>
+          <t xml:space="preserve">sky blue suit</t>
         </is>
       </c>
     </row>
@@ -766,15 +766,15 @@
       </c>
       <c t="inlineStr" r="C12">
         <is>
-          <t xml:space="preserve">sachin</t>
+          <t xml:space="preserve">vignesh</t>
         </is>
       </c>
       <c r="D12" s="65">
-        <v>9895964853</v>
+        <v>8086490774</v>
       </c>
       <c t="inlineStr" r="E12">
         <is>
-          <t xml:space="preserve">30-12-2025</t>
+          <t xml:space="preserve">02-01-2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F12">
@@ -789,12 +789,12 @@
       </c>
       <c t="inlineStr" r="H12">
         <is>
-          <t xml:space="preserve">PRODUCT</t>
+          <t xml:space="preserve">ENQUIRY</t>
         </is>
       </c>
       <c t="inlineStr" r="I12">
         <is>
-          <t xml:space="preserve">PRODUCT NOT AVAILABLE</t>
+          <t xml:space="preserve">ENQUIRY WITHOUT BRIDE/FAMILY</t>
         </is>
       </c>
       <c t="inlineStr" r="J12">
@@ -804,7 +804,7 @@
       </c>
       <c t="inlineStr" r="K12">
         <is>
-          <t xml:space="preserve">sky blue suit</t>
+          <t xml:space="preserve">revist again within 2days</t>
         </is>
       </c>
     </row>
@@ -819,20 +819,20 @@
       </c>
       <c t="inlineStr" r="C13">
         <is>
-          <t xml:space="preserve">vignesh</t>
+          <t xml:space="preserve">shani</t>
         </is>
       </c>
       <c r="D13" s="65">
-        <v>8086490774</v>
+        <v>8281980642</v>
       </c>
       <c t="inlineStr" r="E13">
         <is>
-          <t xml:space="preserve">02-01-2026</t>
+          <t xml:space="preserve">05-01-2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F13">
         <is>
-          <t xml:space="preserve">MUHAMMED ROSHAN C V</t>
+          <t xml:space="preserve">SHAIKRIZWAN</t>
         </is>
       </c>
       <c t="inlineStr" r="G13">
@@ -857,7 +857,7 @@
       </c>
       <c t="inlineStr" r="K13">
         <is>
-          <t xml:space="preserve">revist again within 2days</t>
+          <t xml:space="preserve">need to visit other Store</t>
         </is>
       </c>
     </row>
@@ -867,20 +867,20 @@
       </c>
       <c t="inlineStr" r="B14">
         <is>
-          <t xml:space="preserve">13-12-2025</t>
+          <t xml:space="preserve">14-12-2025</t>
         </is>
       </c>
       <c t="inlineStr" r="C14">
         <is>
-          <t xml:space="preserve">shani</t>
+          <t xml:space="preserve">adarsh</t>
         </is>
       </c>
       <c r="D14" s="65">
-        <v>8281980642</v>
+        <v>7510945212</v>
       </c>
       <c t="inlineStr" r="E14">
         <is>
-          <t xml:space="preserve">05-01-2026</t>
+          <t xml:space="preserve">28-12-2025</t>
         </is>
       </c>
       <c t="inlineStr" r="F14">
@@ -900,7 +900,7 @@
       </c>
       <c t="inlineStr" r="I14">
         <is>
-          <t xml:space="preserve">ENQUIRY WITHOUT BRIDE/FAMILY</t>
+          <t xml:space="preserve">ENQUIRY WITHOUT TRIAL</t>
         </is>
       </c>
       <c t="inlineStr" r="J14">
@@ -910,7 +910,7 @@
       </c>
       <c t="inlineStr" r="K14">
         <is>
-          <t xml:space="preserve">need to visit other Store</t>
+          <t xml:space="preserve">need to visit another store</t>
         </is>
       </c>
     </row>
@@ -925,15 +925,15 @@
       </c>
       <c t="inlineStr" r="C15">
         <is>
-          <t xml:space="preserve">adarsh</t>
+          <t xml:space="preserve">AMJAD</t>
         </is>
       </c>
       <c r="D15" s="65">
-        <v>7510945212</v>
+        <v>8281287445</v>
       </c>
       <c t="inlineStr" r="E15">
         <is>
-          <t xml:space="preserve">28-12-2025</t>
+          <t xml:space="preserve">25-01-2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F15">
@@ -953,7 +953,7 @@
       </c>
       <c t="inlineStr" r="I15">
         <is>
-          <t xml:space="preserve">ENQUIRY WITHOUT TRIAL</t>
+          <t xml:space="preserve">ENQUIRY WITHOUT BRIDE/FAMILY</t>
         </is>
       </c>
       <c t="inlineStr" r="J15">
@@ -963,7 +963,7 @@
       </c>
       <c t="inlineStr" r="K15">
         <is>
-          <t xml:space="preserve">need to visit another store</t>
+          <t xml:space="preserve">WILL VISIT WITH FAMILY MEMBERS</t>
         </is>
       </c>
     </row>
@@ -978,15 +978,15 @@
       </c>
       <c t="inlineStr" r="C16">
         <is>
-          <t xml:space="preserve">AMJAD</t>
+          <t xml:space="preserve">sudin</t>
         </is>
       </c>
       <c r="D16" s="65">
-        <v>8281287445</v>
+        <v>7012152016</v>
       </c>
       <c t="inlineStr" r="E16">
         <is>
-          <t xml:space="preserve">25-01-2026</t>
+          <t xml:space="preserve">04-01-2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F16">
@@ -1006,7 +1006,7 @@
       </c>
       <c t="inlineStr" r="I16">
         <is>
-          <t xml:space="preserve">ENQUIRY WITHOUT BRIDE/FAMILY</t>
+          <t xml:space="preserve">Enquiry for Relative/Friend</t>
         </is>
       </c>
       <c t="inlineStr" r="J16">
@@ -1016,7 +1016,7 @@
       </c>
       <c t="inlineStr" r="K16">
         <is>
-          <t xml:space="preserve">WILL VISIT WITH FAMILY MEMBERS</t>
+          <t xml:space="preserve">revisit again</t>
         </is>
       </c>
     </row>
@@ -1031,15 +1031,15 @@
       </c>
       <c t="inlineStr" r="C17">
         <is>
-          <t xml:space="preserve">sudin</t>
+          <t xml:space="preserve">abu</t>
         </is>
       </c>
       <c r="D17" s="65">
-        <v>7012152016</v>
+        <v>9633673890</v>
       </c>
       <c t="inlineStr" r="E17">
         <is>
-          <t xml:space="preserve">04-01-2026</t>
+          <t xml:space="preserve">21-12-2025</t>
         </is>
       </c>
       <c t="inlineStr" r="F17">
@@ -1059,7 +1059,7 @@
       </c>
       <c t="inlineStr" r="I17">
         <is>
-          <t xml:space="preserve">Enquiry for Relative/Friend</t>
+          <t xml:space="preserve">ENQUIRY WITHOUT BRIDE/FAMILY</t>
         </is>
       </c>
       <c t="inlineStr" r="J17">
@@ -1069,7 +1069,7 @@
       </c>
       <c t="inlineStr" r="K17">
         <is>
-          <t xml:space="preserve">revisit again</t>
+          <t xml:space="preserve">need to visit another store</t>
         </is>
       </c>
     </row>
@@ -1084,20 +1084,20 @@
       </c>
       <c t="inlineStr" r="C18">
         <is>
-          <t xml:space="preserve">abu</t>
+          <t xml:space="preserve">Nithin</t>
         </is>
       </c>
       <c r="D18" s="65">
-        <v>9633673890</v>
+        <v>9188031437</v>
       </c>
       <c t="inlineStr" r="E18">
         <is>
-          <t xml:space="preserve">21-12-2025</t>
+          <t xml:space="preserve">26-01-2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F18">
         <is>
-          <t xml:space="preserve">SHAIKRIZWAN</t>
+          <t xml:space="preserve">RAMITH K</t>
         </is>
       </c>
       <c t="inlineStr" r="G18">
@@ -1112,7 +1112,7 @@
       </c>
       <c t="inlineStr" r="I18">
         <is>
-          <t xml:space="preserve">ENQUIRY WITHOUT BRIDE/FAMILY</t>
+          <t xml:space="preserve">Enquiry for Relative/Friend</t>
         </is>
       </c>
       <c t="inlineStr" r="J18">
@@ -1122,7 +1122,7 @@
       </c>
       <c t="inlineStr" r="K18">
         <is>
-          <t xml:space="preserve">need to visit another store</t>
+          <t xml:space="preserve">Loss</t>
         </is>
       </c>
     </row>
@@ -2766,6 +2766,430 @@
       <c t="inlineStr" r="K49">
         <is>
           <t xml:space="preserve">need to visit other store</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="65">
+        <v>48</v>
+      </c>
+      <c t="inlineStr" r="B50">
+        <is>
+          <t xml:space="preserve">27-12-2025</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C50">
+        <is>
+          <t xml:space="preserve">alan</t>
+        </is>
+      </c>
+      <c r="D50" s="65">
+        <v>7356370841</v>
+      </c>
+      <c t="inlineStr" r="E50">
+        <is>
+          <t xml:space="preserve">13-01-2026</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="F50">
+        <is>
+          <t xml:space="preserve">SHAIKRIZWAN</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="G50">
+        <is>
+          <t xml:space="preserve">Loss</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="H50">
+        <is>
+          <t xml:space="preserve">ENQUIRY</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I50">
+        <is>
+          <t xml:space="preserve">Enquiry for Relative/Friend</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J50">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="K50">
+        <is>
+          <t xml:space="preserve">need to visit another store</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="65">
+        <v>49</v>
+      </c>
+      <c t="inlineStr" r="B51">
+        <is>
+          <t xml:space="preserve">27-12-2025</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C51">
+        <is>
+          <t xml:space="preserve">sreerag</t>
+        </is>
+      </c>
+      <c r="D51" s="65">
+        <v>6238806512</v>
+      </c>
+      <c t="inlineStr" r="E51">
+        <is>
+          <t xml:space="preserve">26-01-2026</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="F51">
+        <is>
+          <t xml:space="preserve">MUHAMMED ROSHAN C V</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="G51">
+        <is>
+          <t xml:space="preserve">Loss</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="H51">
+        <is>
+          <t xml:space="preserve">ENQUIRY</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I51">
+        <is>
+          <t xml:space="preserve">ENQUIRY WITHOUT BRIDE/FAMILY</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J51">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="K51">
+        <is>
+          <t xml:space="preserve">need to visit other stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="65">
+        <v>50</v>
+      </c>
+      <c t="inlineStr" r="B52">
+        <is>
+          <t xml:space="preserve">27-12-2025</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C52">
+        <is>
+          <t xml:space="preserve">ramthushar</t>
+        </is>
+      </c>
+      <c r="D52" s="65">
+        <v>9061123973</v>
+      </c>
+      <c t="inlineStr" r="E52">
+        <is>
+          <t xml:space="preserve">31-12-2025</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="F52">
+        <is>
+          <t xml:space="preserve">SHAIKRIZWAN</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="G52">
+        <is>
+          <t xml:space="preserve">Loss</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="H52">
+        <is>
+          <t xml:space="preserve">ENQUIRY</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I52">
+        <is>
+          <t xml:space="preserve">Enquiry for Relative/Friend</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J52">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="K52">
+        <is>
+          <t xml:space="preserve">revisit again</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="65">
+        <v>51</v>
+      </c>
+      <c t="inlineStr" r="B53">
+        <is>
+          <t xml:space="preserve">28-12-2025</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C53">
+        <is>
+          <t xml:space="preserve">arjun</t>
+        </is>
+      </c>
+      <c r="D53" s="65">
+        <v>9539905435</v>
+      </c>
+      <c t="inlineStr" r="E53">
+        <is>
+          <t xml:space="preserve">14-01-2026</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="F53">
+        <is>
+          <t xml:space="preserve">SHAIKRIZWAN</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="G53">
+        <is>
+          <t xml:space="preserve">Loss</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="H53">
+        <is>
+          <t xml:space="preserve">PRODUCT</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I53">
+        <is>
+          <t xml:space="preserve">PRODUCT NOT AVAILABLE</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J53">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="K53">
+        <is>
+          <t xml:space="preserve">suits collection not okay</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="65">
+        <v>52</v>
+      </c>
+      <c t="inlineStr" r="B54">
+        <is>
+          <t xml:space="preserve">28-12-2025</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C54">
+        <is>
+          <t xml:space="preserve">junaid</t>
+        </is>
+      </c>
+      <c r="D54" s="65">
+        <v>8113936320</v>
+      </c>
+      <c t="inlineStr" r="E54">
+        <is>
+          <t xml:space="preserve">10-01-2026</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="F54">
+        <is>
+          <t xml:space="preserve">AKHIL K</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="G54">
+        <is>
+          <t xml:space="preserve">Loss</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="H54">
+        <is>
+          <t xml:space="preserve">PRODUCT</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I54">
+        <is>
+          <t xml:space="preserve">REQUIRED MODEL NOT AVAILABLE</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J54">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="K54">
+        <is>
+          <t xml:space="preserve">maybe revisit again</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="65">
+        <v>53</v>
+      </c>
+      <c t="inlineStr" r="B55">
+        <is>
+          <t xml:space="preserve">28-12-2025</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C55">
+        <is>
+          <t xml:space="preserve">celes</t>
+        </is>
+      </c>
+      <c r="D55" s="65">
+        <v>8848144289</v>
+      </c>
+      <c t="inlineStr" r="E55">
+        <is>
+          <t xml:space="preserve">07-01-2026</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="F55">
+        <is>
+          <t xml:space="preserve">AKHIL K</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="G55">
+        <is>
+          <t xml:space="preserve">Loss</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="H55">
+        <is>
+          <t xml:space="preserve">ENQUIRY</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I55">
+        <is>
+          <t xml:space="preserve">ENQUIRY WITHOUT BRIDE/FAMILY</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J55">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="K55">
+        <is>
+          <t xml:space="preserve">revisit again</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="65">
+        <v>54</v>
+      </c>
+      <c t="inlineStr" r="B56">
+        <is>
+          <t xml:space="preserve">29-12-2025</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C56">
+        <is>
+          <t xml:space="preserve">akhil</t>
+        </is>
+      </c>
+      <c r="D56" s="65">
+        <v>8139873537</v>
+      </c>
+      <c t="inlineStr" r="E56">
+        <is>
+          <t xml:space="preserve">04-01-2026</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="F56">
+        <is>
+          <t xml:space="preserve">SHAIKRIZWAN</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="G56">
+        <is>
+          <t xml:space="preserve">Loss</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="H56">
+        <is>
+          <t xml:space="preserve">ENQUIRY</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I56">
+        <is>
+          <t xml:space="preserve">ENQUIRY WITHOUT BRIDE/FAMILY</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J56">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="K56">
+        <is>
+          <t xml:space="preserve">need to visit more store</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="65">
+        <v>55</v>
+      </c>
+      <c t="inlineStr" r="B57">
+        <is>
+          <t xml:space="preserve">29-12-2025</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C57">
+        <is>
+          <t xml:space="preserve">rudhbayd</t>
+        </is>
+      </c>
+      <c r="D57" s="65">
+        <v>6238535309</v>
+      </c>
+      <c t="inlineStr" r="E57">
+        <is>
+          <t xml:space="preserve">30-12-2025</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="F57">
+        <is>
+          <t xml:space="preserve">MUHAMMED ROSHAN C V</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="G57">
+        <is>
+          <t xml:space="preserve">Loss</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="H57">
+        <is>
+          <t xml:space="preserve">ENQUIRY</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I57">
+        <is>
+          <t xml:space="preserve">ENQUIRY WITHOUT BRIDE/FAMILY</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J57">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="K57">
+        <is>
+          <t xml:space="preserve">revisit</t>
         </is>
       </c>
     </row>

</xml_diff>